<commit_message>
fix(calculators): fixed double space in name and added stationary fuel values
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/8.2-stationary-fuel.xlsx
+++ b/packages/calculators/src/modules/test/8.2-stationary-fuel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators-internal/packages/calculators/src/modules/test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAC0073-5E8B-904C-A5DE-821A3C7C0ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBC09209-98DC-824A-B255-CD2BA79B00D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51220" yWindow="-4400" windowWidth="28800" windowHeight="19640" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
+    <workbookView xWindow="38400" yWindow="-3000" windowWidth="28800" windowHeight="19640" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="8.2.1.1" sheetId="3" r:id="rId1"/>
@@ -235,9 +235,6 @@
     <t>Other primary solid biomass fuels</t>
   </si>
   <si>
-    <t>Biomass,  municipal and industrial materials</t>
-  </si>
-  <si>
     <t>Scope 1 EF CO2 (kg CO2-e/GJ)</t>
   </si>
   <si>
@@ -502,6 +499,9 @@
   </si>
   <si>
     <t>N2O</t>
+  </si>
+  <si>
+    <t>Biomass, municipal and industrial materials</t>
   </si>
 </sst>
 </file>
@@ -609,8 +609,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -980,7 +980,7 @@
     </row>
     <row r="3" spans="1:26" ht="51">
       <c r="C3" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6" t="s">
@@ -996,12 +996,12 @@
       <c r="N3" s="6"/>
       <c r="O3" s="6"/>
       <c r="P3" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q3" s="6"/>
       <c r="S3" s="1"/>
       <c r="T3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="17">
@@ -1015,7 +1015,7 @@
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E4" t="s">
         <v>5</v>
@@ -1033,7 +1033,7 @@
         <v>9</v>
       </c>
       <c r="J4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K4" t="s">
         <v>15</v>
@@ -1048,13 +1048,13 @@
         <v>17</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="U4">
         <v>28</v>
@@ -1062,7 +1062,7 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
@@ -1071,7 +1071,7 @@
         <v>5</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E5" s="11">
         <f t="shared" ref="E5:E6" si="0">IF(ISBLANK(A5), "", VLOOKUP($B5, _xlfn.IFS($A5="Solid fuels", $S$9:$Z$28,$A5="Cars and light commercial vehicles (pre 2004)", $S$44:$AA$48,$A5="Light duty vehicles",$S$49:$AA$50,$A5="Heavy duty vehicles",$S$51:$AA$58,$A5="Aviation",$S$59:$AA$61,$A5="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -1105,11 +1105,11 @@
         <f t="shared" ref="L5:L6" si="1">C5*E5*G5/1000</f>
         <v>12.15</v>
       </c>
-      <c r="M5" s="16">
+      <c r="M5" s="15">
         <f>(C5*E5*H5/$U$4)/1000</f>
         <v>1.9285714285714286E-4</v>
       </c>
-      <c r="N5" s="16">
+      <c r="N5" s="15">
         <f>(C5*E5*I5/$U$5)/1000</f>
         <v>1.018867924528302E-4</v>
       </c>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="Q5" s="11"/>
       <c r="T5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="U5">
         <v>265</v>
@@ -1131,7 +1131,7 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -1140,7 +1140,7 @@
         <v>6</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E6" s="11">
         <f t="shared" si="0"/>
@@ -1174,11 +1174,11 @@
         <f t="shared" si="1"/>
         <v>11.34</v>
       </c>
-      <c r="M6" s="16">
+      <c r="M6" s="15">
         <f t="shared" ref="M6:M32" si="8">(C6*E6*H6/$U$4)/1000</f>
         <v>1.7999999999999998E-4</v>
       </c>
-      <c r="N6" s="16">
+      <c r="N6" s="15">
         <f t="shared" ref="N6:N32" si="9">(C6*E6*I6/$U$5)/1000</f>
         <v>9.5094339622641528E-5</v>
       </c>
@@ -1194,7 +1194,7 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
         <v>22</v>
@@ -1203,7 +1203,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E7" s="11">
         <f>IF(ISBLANK(A7), "", VLOOKUP($B7, _xlfn.IFS($A7="Solid fuels", $S$9:$Z$28,$A7="Cars and light commercial vehicles (pre 2004)", $S$44:$AA$48,$A7="Light duty vehicles",$S$49:$AA$50,$A7="Heavy duty vehicles",$S$51:$AA$58,$A7="Aviation",$S$59:$AA$61,$A7="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -1237,11 +1237,11 @@
         <f t="shared" ref="L7:L26" si="12">C7*E7*G7/1000</f>
         <v>7.629599999999999</v>
       </c>
-      <c r="M7" s="16">
+      <c r="M7" s="15">
         <f t="shared" si="8"/>
         <v>5.8285714285714284E-5</v>
       </c>
-      <c r="N7" s="16">
+      <c r="N7" s="15">
         <f t="shared" si="9"/>
         <v>9.2377358490566022E-5</v>
       </c>
@@ -1257,7 +1257,7 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
         <v>23</v>
@@ -1266,7 +1266,7 @@
         <v>9</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E8" s="11">
         <f>IF(ISBLANK(A8), "", VLOOKUP($B8, _xlfn.IFS($A8="Solid fuels", $S$9:$Z$28,$A8="Cars and light commercial vehicles (pre 2004)", $S$44:$AA$48,$A8="Light duty vehicles",$S$49:$AA$50,$A8="Heavy duty vehicles",$S$51:$AA$58,$A8="Aviation",$S$59:$AA$61,$A8="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -1300,11 +1300,11 @@
         <f t="shared" si="12"/>
         <v>24.786000000000001</v>
       </c>
-      <c r="M8" s="16">
+      <c r="M8" s="15">
         <f t="shared" si="8"/>
         <v>2.8928571428571425E-4</v>
       </c>
-      <c r="N8" s="16">
+      <c r="N8" s="15">
         <f t="shared" si="9"/>
         <v>2.0377358490566039E-4</v>
       </c>
@@ -1324,36 +1324,36 @@
         <v>18</v>
       </c>
       <c r="U8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="V8" t="s">
+        <v>38</v>
+      </c>
+      <c r="W8" t="s">
         <v>39</v>
       </c>
-      <c r="W8" t="s">
+      <c r="X8" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>93</v>
+      </c>
+      <c r="Z8" t="s">
         <v>40</v>
-      </c>
-      <c r="X8" t="s">
-        <v>93</v>
-      </c>
-      <c r="Y8" t="s">
-        <v>94</v>
-      </c>
-      <c r="Z8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:26">
       <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s">
         <v>43</v>
-      </c>
-      <c r="B9" t="s">
-        <v>44</v>
       </c>
       <c r="C9">
         <v>8</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E9" s="11">
         <f t="shared" ref="E9:E16" si="14">IF(ISBLANK(A9), "", VLOOKUP($B9, _xlfn.IFS($A9="Solid fuels", $S$9:$Z$28,$A9="Liquid fuels", $S$29:$Z$39,$A9="Light duty vehicles",$S$49:$AA$50,$A9="Heavy duty vehicles",$S$51:$AA$58,$A9="Aviation",$S$59:$AA$61,$A9="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -1387,11 +1387,11 @@
         <f t="shared" si="12"/>
         <v>4.3145599999999993</v>
       </c>
-      <c r="M9" s="16">
+      <c r="M9" s="15">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="N9" s="16">
+      <c r="N9" s="15">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="Q9" s="11"/>
       <c r="R9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S9" t="s">
         <v>19</v>
@@ -1414,7 +1414,7 @@
         <v>27</v>
       </c>
       <c r="U9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V9">
         <v>90</v>
@@ -1434,16 +1434,16 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C10">
         <v>9</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E10" s="11">
         <f t="shared" si="14"/>
@@ -1477,11 +1477,11 @@
         <f t="shared" si="12"/>
         <v>1.2222</v>
       </c>
-      <c r="M10" s="16">
+      <c r="M10" s="15">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="N10" s="16">
+      <c r="N10" s="15">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>21</v>
       </c>
       <c r="U10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V10">
         <v>90</v>
@@ -1521,16 +1521,16 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11">
         <v>12</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E11" s="11">
         <f t="shared" si="14"/>
@@ -1564,11 +1564,11 @@
         <f t="shared" si="12"/>
         <v>27.660960000000006</v>
       </c>
-      <c r="M11" s="16">
+      <c r="M11" s="15">
         <f t="shared" si="8"/>
         <v>2.9314285714285718E-3</v>
       </c>
-      <c r="N11" s="16">
+      <c r="N11" s="15">
         <f t="shared" si="9"/>
         <v>3.0973584905660383E-4</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>29</v>
       </c>
       <c r="U11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V11">
         <v>90</v>
@@ -1603,21 +1603,21 @@
         <v>90.24</v>
       </c>
       <c r="Z11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:26">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C12">
         <v>13</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E12" s="11">
         <f t="shared" si="14"/>
@@ -1651,11 +1651,11 @@
         <f t="shared" si="12"/>
         <v>28.830100000000002</v>
       </c>
-      <c r="M12" s="16">
+      <c r="M12" s="15">
         <f t="shared" si="8"/>
         <v>3.073571428571429E-3</v>
       </c>
-      <c r="N12" s="16">
+      <c r="N12" s="15">
         <f t="shared" si="9"/>
         <v>3.2475471698113209E-4</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>10.199999999999999</v>
       </c>
       <c r="U12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V12">
         <v>93.5</v>
@@ -1695,16 +1695,16 @@
     </row>
     <row r="13" spans="1:26" ht="17">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C13">
         <v>14</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E13" s="11">
         <f t="shared" si="14"/>
@@ -1738,11 +1738,11 @@
         <f t="shared" si="12"/>
         <v>36.172499999999999</v>
       </c>
-      <c r="M13" s="16">
+      <c r="M13" s="15">
         <f t="shared" si="8"/>
         <v>1.875E-4</v>
       </c>
-      <c r="N13" s="16">
+      <c r="N13" s="15">
         <f t="shared" si="9"/>
         <v>3.9622641509433966E-4</v>
       </c>
@@ -1762,7 +1762,7 @@
         <v>30</v>
       </c>
       <c r="U13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V13">
         <v>91.8</v>
@@ -1782,16 +1782,16 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14">
         <v>15</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E14" s="11">
         <f t="shared" si="14"/>
@@ -1825,11 +1825,11 @@
         <f t="shared" si="12"/>
         <v>38.419199999999996</v>
       </c>
-      <c r="M14" s="16">
+      <c r="M14" s="15">
         <f t="shared" si="8"/>
         <v>3.9428571428571431E-4</v>
       </c>
-      <c r="N14" s="16">
+      <c r="N14" s="15">
         <f t="shared" si="9"/>
         <v>4.166037735849057E-4</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>22.1</v>
       </c>
       <c r="U14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V14">
         <v>95</v>
@@ -1864,21 +1864,21 @@
         <v>95.38</v>
       </c>
       <c r="Z14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:26">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15">
         <v>16</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E15" s="11">
         <f t="shared" si="14"/>
@@ -1912,11 +1912,11 @@
         <f t="shared" si="12"/>
         <v>41.477599999999995</v>
       </c>
-      <c r="M15" s="16">
+      <c r="M15" s="15">
         <f t="shared" si="8"/>
         <v>6.3942857142857139E-4</v>
       </c>
-      <c r="N15" s="16">
+      <c r="N15" s="15">
         <f t="shared" si="9"/>
         <v>4.5041509433962261E-4</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>27</v>
       </c>
       <c r="U15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V15">
         <v>107</v>
@@ -1951,12 +1951,12 @@
         <v>107.23</v>
       </c>
       <c r="Z15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:26">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" t="s">
         <v>11</v>
@@ -1965,7 +1965,7 @@
         <v>17</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E16" s="11">
         <f t="shared" si="14"/>
@@ -1999,11 +1999,11 @@
         <f t="shared" si="12"/>
         <v>45.868380000000002</v>
       </c>
-      <c r="M16" s="16">
+      <c r="M16" s="15">
         <f t="shared" si="8"/>
         <v>2.3435714285714288E-3</v>
       </c>
-      <c r="N16" s="16">
+      <c r="N16" s="15">
         <f t="shared" si="9"/>
         <v>4.9524528301886795E-4</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>37.5</v>
       </c>
       <c r="U16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V16">
         <v>81.8</v>
@@ -2038,12 +2038,12 @@
         <v>82.03</v>
       </c>
       <c r="Z16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:26">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
@@ -2052,7 +2052,7 @@
         <v>18</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E17" s="11">
         <f t="shared" ref="E17:E25" si="21">IF(ISBLANK(A17), "", VLOOKUP($B17, _xlfn.IFS($A17="Solid fuels", $S$9:$Z$28,$A17="Liquid fuels", $S$29:$Z$52,$A17="Light duty vehicles",$S$49:$AA$50,$A17="Heavy duty vehicles",$S$51:$AA$58,$A17="Aviation",$S$59:$AA$61,$A17="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -2086,11 +2086,11 @@
         <f t="shared" si="12"/>
         <v>52.594559999999994</v>
       </c>
-      <c r="M17" s="16">
+      <c r="M17" s="15">
         <f t="shared" si="8"/>
         <v>1.020857142857143E-3</v>
       </c>
-      <c r="N17" s="16">
+      <c r="N17" s="15">
         <f t="shared" si="9"/>
         <v>5.3932075471698111E-4</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>22.1</v>
       </c>
       <c r="U17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V17">
         <v>95</v>
@@ -2125,21 +2125,21 @@
         <v>95.28</v>
       </c>
       <c r="Z17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:26">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C18">
         <v>17</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E18" s="11">
         <f t="shared" si="21"/>
@@ -2173,11 +2173,11 @@
         <f t="shared" si="12"/>
         <v>40.760559999999998</v>
       </c>
-      <c r="M18" s="16">
+      <c r="M18" s="15">
         <f t="shared" si="8"/>
         <v>6.2657142857142848E-4</v>
       </c>
-      <c r="N18" s="16">
+      <c r="N18" s="15">
         <f t="shared" si="9"/>
         <v>4.413584905660377E-4</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>26.3</v>
       </c>
       <c r="U18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V18">
         <v>81.599999999999994</v>
@@ -2212,21 +2212,21 @@
         <v>81.83</v>
       </c>
       <c r="Z18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:26">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C19">
         <v>16</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E19" s="11">
         <f t="shared" si="21"/>
@@ -2260,11 +2260,11 @@
         <f t="shared" si="12"/>
         <v>38.362879999999997</v>
       </c>
-      <c r="M19" s="16">
+      <c r="M19" s="15">
         <f t="shared" si="8"/>
         <v>5.8971428571428575E-4</v>
       </c>
-      <c r="N19" s="16">
+      <c r="N19" s="15">
         <f t="shared" si="9"/>
         <v>4.1539622641509431E-4</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>32</v>
       </c>
       <c r="U19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V19">
         <v>62.8</v>
@@ -2299,21 +2299,21 @@
         <v>63.03</v>
       </c>
       <c r="Z19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:26">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C20">
         <v>15</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E20" s="11">
         <f t="shared" si="21"/>
@@ -2347,11 +2347,11 @@
         <f t="shared" si="12"/>
         <v>23.207100000000001</v>
       </c>
-      <c r="M20" s="16">
+      <c r="M20" s="15">
         <f t="shared" si="8"/>
         <v>2.753571428571429E-3</v>
       </c>
-      <c r="N20" s="16">
+      <c r="N20" s="15">
         <f t="shared" si="9"/>
         <v>2.9094339622641512E-4</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>27.1</v>
       </c>
       <c r="U20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V20">
         <v>55.9</v>
@@ -2386,21 +2386,21 @@
         <v>56.13</v>
       </c>
       <c r="Z20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:26">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C21">
         <v>14</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E21" s="11">
         <f t="shared" si="21"/>
@@ -2434,11 +2434,11 @@
         <f t="shared" si="12"/>
         <v>30.684079999999998</v>
       </c>
-      <c r="M21" s="16">
+      <c r="M21" s="15">
         <f t="shared" si="8"/>
         <v>1.5699999999999999E-4</v>
       </c>
-      <c r="N21" s="16">
+      <c r="N21" s="15">
         <f t="shared" si="9"/>
         <v>1.6588679245283017E-5</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>10.5</v>
       </c>
       <c r="U21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V21">
         <v>87.1</v>
@@ -2473,21 +2473,21 @@
         <v>88.9</v>
       </c>
       <c r="Z21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:26">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C22">
         <v>13</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E22" s="11">
         <f t="shared" si="21"/>
@@ -2521,11 +2521,11 @@
         <f t="shared" si="12"/>
         <v>41.169959999999996</v>
       </c>
-      <c r="M22" s="16">
+      <c r="M22" s="15">
         <f t="shared" si="8"/>
         <v>1.2702857142857145E-3</v>
       </c>
-      <c r="N22" s="16">
+      <c r="N22" s="15">
         <f t="shared" si="9"/>
         <v>3.3554716981132083E-4</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>16.2</v>
       </c>
       <c r="U22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V22">
         <v>0</v>
@@ -2560,21 +2560,21 @@
         <v>1.2</v>
       </c>
       <c r="Z22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:26">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C23">
         <v>12</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E23" s="11">
         <f t="shared" si="21"/>
@@ -2608,11 +2608,11 @@
         <f t="shared" si="12"/>
         <v>28.159559999999999</v>
       </c>
-      <c r="M23" s="16">
+      <c r="M23" s="15">
         <f t="shared" si="8"/>
         <v>5.515714285714285E-4</v>
       </c>
-      <c r="N23" s="16">
+      <c r="N23" s="15">
         <f t="shared" si="9"/>
         <v>5.827924528301886E-5</v>
       </c>
@@ -2632,7 +2632,7 @@
         <v>10.4</v>
       </c>
       <c r="U23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V23">
         <v>0</v>
@@ -2647,21 +2647,21 @@
         <v>1.2</v>
       </c>
       <c r="Z23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:26">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C24">
         <v>11</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E24" s="11">
         <f t="shared" si="21"/>
@@ -2695,11 +2695,11 @@
         <f t="shared" si="12"/>
         <v>34.836120000000001</v>
       </c>
-      <c r="M24" s="16">
+      <c r="M24" s="15">
         <f t="shared" si="8"/>
         <v>1.074857142857143E-3</v>
       </c>
-      <c r="N24" s="16">
+      <c r="N24" s="15">
         <f t="shared" si="9"/>
         <v>2.8392452830188679E-4</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>12.4</v>
       </c>
       <c r="U24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V24" s="2">
         <v>0</v>
@@ -2734,21 +2734,21 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="Z24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:26">
       <c r="A25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C25">
         <v>10</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25" s="11">
         <f t="shared" si="21"/>
@@ -2782,11 +2782,11 @@
         <f t="shared" si="12"/>
         <v>24.011200000000002</v>
       </c>
-      <c r="M25" s="16">
+      <c r="M25" s="15">
         <f t="shared" si="8"/>
         <v>2.4571428571428574E-4</v>
       </c>
-      <c r="N25" s="16">
+      <c r="N25" s="15">
         <f t="shared" si="9"/>
         <v>1.2981132075471697E-4</v>
       </c>
@@ -2806,7 +2806,7 @@
         <v>9.6</v>
       </c>
       <c r="U25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V25" s="2">
         <v>0</v>
@@ -2821,21 +2821,21 @@
         <v>1.4</v>
       </c>
       <c r="Z25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:26">
       <c r="A26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" t="s">
         <v>56</v>
-      </c>
-      <c r="B26" t="s">
-        <v>57</v>
       </c>
       <c r="C26">
         <v>6</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E26" s="11">
         <f t="shared" ref="E26:E32" si="27">$T$53</f>
@@ -2869,11 +2869,11 @@
         <f t="shared" si="12"/>
         <v>7.8025200000000003</v>
       </c>
-      <c r="M26" s="16">
+      <c r="M26" s="15">
         <f t="shared" si="8"/>
         <v>5.4214285714285714E-4</v>
       </c>
-      <c r="N26" s="16">
+      <c r="N26" s="15">
         <f t="shared" si="9"/>
         <v>1.7184905660377361E-5</v>
       </c>
@@ -2887,13 +2887,13 @@
       </c>
       <c r="Q26" s="11"/>
       <c r="S26" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="T26" s="2">
         <v>12.2</v>
       </c>
       <c r="U26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V26">
         <v>0</v>
@@ -2908,21 +2908,21 @@
         <v>1.8</v>
       </c>
       <c r="Z26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:26">
       <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="s">
         <v>56</v>
-      </c>
-      <c r="B27" t="s">
-        <v>57</v>
       </c>
       <c r="C27">
         <v>7</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E27" s="11">
         <f t="shared" si="27"/>
@@ -2956,11 +2956,11 @@
         <f t="shared" ref="L27:L29" si="34">C27*E27*G27/1000</f>
         <v>9.1029399999999985</v>
       </c>
-      <c r="M27" s="16">
+      <c r="M27" s="15">
         <f t="shared" si="8"/>
         <v>6.3250000000000003E-4</v>
       </c>
-      <c r="N27" s="16">
+      <c r="N27" s="15">
         <f t="shared" si="9"/>
         <v>2.0049056603773583E-5</v>
       </c>
@@ -2980,7 +2980,7 @@
         <v>31.1</v>
       </c>
       <c r="U27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V27" s="2">
         <v>0</v>
@@ -2995,21 +2995,21 @@
         <v>6.3</v>
       </c>
       <c r="Z27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:26">
       <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
         <v>56</v>
-      </c>
-      <c r="B28" t="s">
-        <v>57</v>
       </c>
       <c r="C28">
         <v>8</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E28" s="11">
         <f t="shared" si="27"/>
@@ -3043,11 +3043,11 @@
         <f t="shared" si="34"/>
         <v>10.403360000000001</v>
       </c>
-      <c r="M28" s="16">
+      <c r="M28" s="15">
         <f t="shared" si="8"/>
         <v>7.2285714285714293E-4</v>
       </c>
-      <c r="N28" s="16">
+      <c r="N28" s="15">
         <f t="shared" si="9"/>
         <v>2.2913207547169811E-5</v>
       </c>
@@ -3067,7 +3067,7 @@
         <v>12.2</v>
       </c>
       <c r="U28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V28" s="2">
         <v>0</v>
@@ -3082,21 +3082,21 @@
         <v>1.8</v>
       </c>
       <c r="Z28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:26">
       <c r="A29" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" t="s">
         <v>56</v>
-      </c>
-      <c r="B29" t="s">
-        <v>57</v>
       </c>
       <c r="C29">
         <v>9</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E29" s="11">
         <f t="shared" si="27"/>
@@ -3130,11 +3130,11 @@
         <f t="shared" si="34"/>
         <v>11.70378</v>
       </c>
-      <c r="M29" s="16">
+      <c r="M29" s="15">
         <f t="shared" si="8"/>
         <v>8.1321428571428582E-4</v>
       </c>
-      <c r="N29" s="16">
+      <c r="N29" s="15">
         <f t="shared" si="9"/>
         <v>2.577735849056604E-5</v>
       </c>
@@ -3148,10 +3148,10 @@
       </c>
       <c r="Q29" s="11"/>
       <c r="R29" t="s">
+        <v>42</v>
+      </c>
+      <c r="S29" t="s">
         <v>43</v>
-      </c>
-      <c r="S29" t="s">
-        <v>44</v>
       </c>
       <c r="T29" s="2">
         <v>38.799999999999997</v>
@@ -3177,16 +3177,16 @@
     </row>
     <row r="30" spans="1:26">
       <c r="A30" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" t="s">
         <v>56</v>
-      </c>
-      <c r="B30" t="s">
-        <v>57</v>
       </c>
       <c r="C30">
         <v>11</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E30" s="11">
         <f t="shared" si="27"/>
@@ -3220,11 +3220,11 @@
         <f>C30*E30*G30/1000</f>
         <v>14.304620000000002</v>
       </c>
-      <c r="M30" s="16">
+      <c r="M30" s="15">
         <f t="shared" si="8"/>
         <v>9.9392857142857139E-4</v>
       </c>
-      <c r="N30" s="16">
+      <c r="N30" s="15">
         <f t="shared" si="9"/>
         <v>3.1505660377358487E-5</v>
       </c>
@@ -3238,7 +3238,7 @@
       </c>
       <c r="Q30" s="11"/>
       <c r="S30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="T30">
         <v>38.799999999999997</v>
@@ -3264,16 +3264,16 @@
     </row>
     <row r="31" spans="1:26">
       <c r="A31" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" t="s">
         <v>56</v>
-      </c>
-      <c r="B31" t="s">
-        <v>57</v>
       </c>
       <c r="C31">
         <v>12</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E31" s="11">
         <f t="shared" si="27"/>
@@ -3307,11 +3307,11 @@
         <f t="shared" ref="L31:L32" si="35">C31*E31*G31/1000</f>
         <v>15.605040000000001</v>
       </c>
-      <c r="M31" s="16">
+      <c r="M31" s="15">
         <f t="shared" si="8"/>
         <v>1.0842857142857143E-3</v>
       </c>
-      <c r="N31" s="16">
+      <c r="N31" s="15">
         <f t="shared" si="9"/>
         <v>3.4369811320754722E-5</v>
       </c>
@@ -3325,13 +3325,13 @@
       </c>
       <c r="Q31" s="11"/>
       <c r="S31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T31" s="2">
         <v>45.3</v>
       </c>
       <c r="U31" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V31" s="2">
         <v>69.599999999999994</v>
@@ -3346,21 +3346,21 @@
         <v>69.88</v>
       </c>
       <c r="Z31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:26">
       <c r="A32" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32" t="s">
         <v>56</v>
-      </c>
-      <c r="B32" t="s">
-        <v>57</v>
       </c>
       <c r="C32">
         <v>13</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E32" s="11">
         <f t="shared" si="27"/>
@@ -3394,11 +3394,11 @@
         <f t="shared" si="35"/>
         <v>16.905460000000001</v>
       </c>
-      <c r="M32" s="16">
+      <c r="M32" s="15">
         <f t="shared" si="8"/>
         <v>1.1746428571428574E-3</v>
       </c>
-      <c r="N32" s="16">
+      <c r="N32" s="15">
         <f t="shared" si="9"/>
         <v>3.7233962264150944E-5</v>
       </c>
@@ -3412,13 +3412,13 @@
       </c>
       <c r="Q32" s="11"/>
       <c r="S32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="T32" s="2">
         <v>46.5</v>
       </c>
       <c r="U32" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V32" s="2">
         <v>61</v>
@@ -3433,13 +3433,13 @@
         <v>61.28</v>
       </c>
       <c r="Z32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:32">
       <c r="Q33" s="11"/>
       <c r="S33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="T33">
         <v>34.200000000000003</v>
@@ -3466,7 +3466,7 @@
     <row r="34" spans="1:32">
       <c r="Q34" s="11"/>
       <c r="S34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="T34" s="2">
         <v>33.1</v>
@@ -3494,7 +3494,7 @@
       <c r="Q35" s="11"/>
       <c r="R35" s="6"/>
       <c r="S35" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="T35" s="13">
         <v>37.5</v>
@@ -3518,8 +3518,8 @@
         <v>18</v>
       </c>
       <c r="AA35" s="6"/>
-      <c r="AC35" s="15" t="s">
-        <v>58</v>
+      <c r="AC35" s="16" t="s">
+        <v>57</v>
       </c>
       <c r="AD35" s="2"/>
       <c r="AE35" s="2"/>
@@ -3527,7 +3527,7 @@
     <row r="36" spans="1:32" ht="34">
       <c r="Q36" s="11"/>
       <c r="S36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="T36" s="2">
         <v>36.799999999999997</v>
@@ -3550,21 +3550,21 @@
       <c r="Z36">
         <v>18</v>
       </c>
-      <c r="AC36" s="15"/>
+      <c r="AC36" s="16"/>
       <c r="AD36" s="13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AE36" s="13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AF36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37" spans="1:32">
       <c r="Q37" s="11"/>
       <c r="S37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="T37">
         <v>37.299999999999997</v>
@@ -3587,12 +3587,12 @@
       <c r="Z37">
         <v>18</v>
       </c>
-      <c r="AC37" s="15"/>
+      <c r="AC37" s="16"/>
       <c r="AD37" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AE37" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="AE37" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:32">
@@ -3622,10 +3622,10 @@
         <v>17.3</v>
       </c>
       <c r="AC38" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AD38" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AE38" s="2">
         <v>14</v>
@@ -3633,7 +3633,7 @@
     </row>
     <row r="39" spans="1:32">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="Q39" s="11"/>
       <c r="S39" t="s">
@@ -3661,10 +3661,10 @@
         <v>18</v>
       </c>
       <c r="AC39" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AD39" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AE39" s="2">
         <v>4</v>
@@ -3672,7 +3672,7 @@
     </row>
     <row r="40" spans="1:32">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B40" t="s">
         <v>21</v>
@@ -3681,7 +3681,7 @@
         <v>7</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E40" s="11">
         <f t="shared" ref="E40:E55" si="36">IF(ISBLANK(A40), "", VLOOKUP($B40, _xlfn.IFS($A40="Solid fuels", $S$9:$Z$28,$A40="Cars and light commercial vehicles (pre 2004)", $S$44:$AA$48,$A40="Light duty vehicles",$S$49:$AA$50,$A40="Heavy duty vehicles",$S$51:$AA$58,$A40="Aviation",$S$59:$AA$61,$A40="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="Q40" s="11"/>
       <c r="S40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="T40">
         <v>34.4</v>
@@ -3751,10 +3751,10 @@
         <v>18</v>
       </c>
       <c r="AC40" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AD40" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AE40" s="2">
         <v>7.9</v>
@@ -3762,7 +3762,7 @@
     </row>
     <row r="41" spans="1:32">
       <c r="A41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41" t="s">
         <v>24</v>
@@ -3771,7 +3771,7 @@
         <v>10</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E41" s="11">
         <f t="shared" si="36"/>
@@ -3817,7 +3817,7 @@
       </c>
       <c r="Q41" s="11"/>
       <c r="S41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="T41" s="2">
         <v>34.4</v>
@@ -3841,10 +3841,10 @@
         <v>18</v>
       </c>
       <c r="AC41" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AD41" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AE41" s="2">
         <v>10.6</v>
@@ -3852,7 +3852,7 @@
     </row>
     <row r="42" spans="1:32">
       <c r="A42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
         <v>25</v>
@@ -3861,7 +3861,7 @@
         <v>11</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E42" s="11">
         <f t="shared" si="36"/>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="Q42" s="11"/>
       <c r="S42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="T42" s="2">
         <v>25.7</v>
@@ -3933,10 +3933,10 @@
       <c r="AA42" s="9"/>
       <c r="AB42" s="9"/>
       <c r="AC42" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AD42" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AE42" s="2">
         <v>4</v>
@@ -3944,7 +3944,7 @@
     </row>
     <row r="43" spans="1:32">
       <c r="A43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" t="s">
         <v>26</v>
@@ -3953,7 +3953,7 @@
         <v>12</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E43" s="11">
         <f t="shared" si="36"/>
@@ -3998,7 +3998,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S43" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="T43" s="2">
         <v>31.4</v>
@@ -4024,7 +4024,7 @@
       <c r="AA43" s="9"/>
       <c r="AB43" s="9"/>
       <c r="AC43" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AD43" s="2" t="str">
         <f>AD39</f>
@@ -4037,7 +4037,7 @@
     </row>
     <row r="44" spans="1:32">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B44" t="s">
         <v>27</v>
@@ -4046,7 +4046,7 @@
         <v>4</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E44" s="11">
         <f t="shared" si="36"/>
@@ -4091,13 +4091,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="S44" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="T44" s="2">
         <v>34.200000000000003</v>
       </c>
       <c r="U44" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V44">
         <v>92.6</v>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="AB44" s="9"/>
       <c r="AC44" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AD44" s="2" t="str">
         <f>AD42</f>
@@ -4129,7 +4129,7 @@
     </row>
     <row r="45" spans="1:32">
       <c r="A45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B45" t="s">
         <v>28</v>
@@ -4138,7 +4138,7 @@
         <v>6</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E45" s="11">
         <f t="shared" si="36"/>
@@ -4183,13 +4183,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="S45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T45">
         <v>42.9</v>
       </c>
       <c r="U45" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V45">
         <v>54.7</v>
@@ -4210,7 +4210,7 @@
     </row>
     <row r="46" spans="1:32">
       <c r="A46" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B46" t="s">
         <v>29</v>
@@ -4219,7 +4219,7 @@
         <v>7</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E46" s="11">
         <f t="shared" si="36"/>
@@ -4264,13 +4264,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="S46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="T46" s="2">
         <v>34.200000000000003</v>
       </c>
       <c r="U46" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V46">
         <v>92.6</v>
@@ -4292,7 +4292,7 @@
     </row>
     <row r="47" spans="1:32">
       <c r="A47" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B47" t="s">
         <v>30</v>
@@ -4301,7 +4301,7 @@
         <v>8</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E47" s="11">
         <f t="shared" si="36"/>
@@ -4346,7 +4346,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S47" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="T47" s="2">
         <v>34.4</v>
@@ -4374,7 +4374,7 @@
     </row>
     <row r="48" spans="1:32">
       <c r="A48" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B48" t="s">
         <v>31</v>
@@ -4383,7 +4383,7 @@
         <v>7</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E48" s="11">
         <f t="shared" si="36"/>
@@ -4428,7 +4428,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S48" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="T48" s="2">
         <v>34.6</v>
@@ -4449,7 +4449,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="Z48" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA48" s="9"/>
       <c r="AB48" s="9"/>
@@ -4457,7 +4457,7 @@
     </row>
     <row r="49" spans="1:29">
       <c r="A49" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B49" t="s">
         <v>32</v>
@@ -4466,7 +4466,7 @@
         <v>8</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E49" s="11">
         <f t="shared" si="36"/>
@@ -4511,7 +4511,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S49" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="T49" s="2">
         <v>23.4</v>
@@ -4532,7 +4532,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="Z49" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA49" s="9"/>
       <c r="AB49" s="9"/>
@@ -4540,7 +4540,7 @@
     </row>
     <row r="50" spans="1:29">
       <c r="A50" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B50" t="s">
         <v>33</v>
@@ -4549,7 +4549,7 @@
         <v>9</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E50" s="11">
         <f t="shared" si="36"/>
@@ -4594,7 +4594,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T50" s="2">
         <v>23.4</v>
@@ -4615,7 +4615,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="Z50" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA50" s="9"/>
       <c r="AB50" s="9"/>
@@ -4623,7 +4623,7 @@
     </row>
     <row r="51" spans="1:29">
       <c r="A51" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B51" t="s">
         <v>34</v>
@@ -4632,7 +4632,7 @@
         <v>10</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E51" s="11">
         <f t="shared" si="36"/>
@@ -4677,7 +4677,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S51" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="T51" s="2">
         <v>36.799999999999997</v>
@@ -4698,7 +4698,7 @@
         <v>0.22</v>
       </c>
       <c r="Z51" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA51" s="9"/>
       <c r="AB51" s="9"/>
@@ -4706,7 +4706,7 @@
     </row>
     <row r="52" spans="1:29">
       <c r="A52" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B52" t="s">
         <v>35</v>
@@ -4715,7 +4715,7 @@
         <v>11</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E52" s="11">
         <f t="shared" si="36"/>
@@ -4760,7 +4760,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="S52" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T52">
         <v>38.6</v>
@@ -4781,7 +4781,7 @@
         <v>0.3</v>
       </c>
       <c r="Z52" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA52" s="9"/>
       <c r="AB52" s="9"/>
@@ -4789,16 +4789,16 @@
     </row>
     <row r="53" spans="1:29">
       <c r="A53" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="C53">
         <v>12</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E53" s="11">
         <f t="shared" si="36"/>
@@ -4843,10 +4843,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="R53" t="s">
+        <v>55</v>
+      </c>
+      <c r="S53" t="s">
         <v>56</v>
-      </c>
-      <c r="S53" t="s">
-        <v>57</v>
       </c>
       <c r="T53" s="2">
         <v>25.3</v>
@@ -4874,7 +4874,7 @@
     </row>
     <row r="54" spans="1:29">
       <c r="A54" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B54" t="s">
         <v>36</v>
@@ -4883,7 +4883,7 @@
         <v>13</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E54" s="11">
         <f t="shared" si="36"/>
@@ -4939,7 +4939,7 @@
     </row>
     <row r="55" spans="1:29">
       <c r="A55" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B55" t="s">
         <v>37</v>
@@ -4948,7 +4948,7 @@
         <v>8</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E55" s="11">
         <f t="shared" si="36"/>
@@ -5004,16 +5004,16 @@
     </row>
     <row r="56" spans="1:29">
       <c r="A56" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B56" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C56">
         <v>10</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E56" s="11">
         <f>IF(ISBLANK(A56), "", VLOOKUP($B56, _xlfn.IFS($A56="Solid fuels", $S$9:$Z$28,$A56="Liquid fuels", $S$29:$Z$39,$A56="Light duty vehicles",$S$49:$AA$50,$A56="Heavy duty vehicles",$S$51:$AA$58,$A56="Aviation",$S$59:$AA$61,$A56="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -5069,16 +5069,16 @@
     </row>
     <row r="57" spans="1:29">
       <c r="A57" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B57" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C57">
         <v>11</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E57" s="11">
         <f>IF(ISBLANK(A57), "", VLOOKUP($B57, _xlfn.IFS($A57="Solid fuels", $S$9:$Z$28,$A57="Liquid fuels", $S$29:$Z$39,$A57="Light duty vehicles",$S$49:$AA$50,$A57="Heavy duty vehicles",$S$51:$AA$58,$A57="Aviation",$S$59:$AA$61,$A57="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -5134,16 +5134,16 @@
     </row>
     <row r="58" spans="1:29">
       <c r="A58" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C58">
         <v>9</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E58" s="11">
         <f>IF(ISBLANK(A58), "", VLOOKUP($B58, _xlfn.IFS($A58="Solid fuels", $S$9:$Z$28,$A58="Liquid fuels", $S$29:$Z$52,$A58="Light duty vehicles",$S$49:$AA$50,$A58="Heavy duty vehicles",$S$51:$AA$58,$A58="Aviation",$S$59:$AA$61,$A58="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -5199,16 +5199,16 @@
     </row>
     <row r="59" spans="1:29">
       <c r="A59" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B59" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C59">
         <v>8</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E59" s="11">
         <f>IF(ISBLANK(A59), "", VLOOKUP($B59, _xlfn.IFS($A59="Solid fuels", $S$9:$Z$28,$A59="Liquid fuels", $S$29:$Z$52,$A59="Light duty vehicles",$S$49:$AA$50,$A59="Heavy duty vehicles",$S$51:$AA$58,$A59="Aviation",$S$59:$AA$61,$A59="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -5264,16 +5264,16 @@
     </row>
     <row r="60" spans="1:29">
       <c r="A60" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B60" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C60">
         <v>7</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E60" s="11">
         <f>IF(ISBLANK(A60), "", VLOOKUP($B60, _xlfn.IFS($A60="Solid fuels", $S$9:$Z$28,$A60="Liquid fuels", $S$29:$Z$52,$A60="Light duty vehicles",$S$49:$AA$50,$A60="Heavy duty vehicles",$S$51:$AA$58,$A60="Aviation",$S$59:$AA$61,$A60="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -5329,16 +5329,16 @@
     </row>
     <row r="61" spans="1:29">
       <c r="A61" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C61">
         <v>6</v>
       </c>
       <c r="D61" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E61" s="11">
         <f>IF(ISBLANK(A61), "", VLOOKUP($B61, _xlfn.IFS($A61="Solid fuels", $S$9:$Z$28,$A61="Liquid fuels", $S$29:$Z$52,$A61="Light duty vehicles",$S$49:$AA$50,$A61="Heavy duty vehicles",$S$51:$AA$58,$A61="Aviation",$S$59:$AA$61,$A61="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>
@@ -5394,16 +5394,16 @@
     </row>
     <row r="62" spans="1:29">
       <c r="A62" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B62" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C62">
         <v>5</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E62" s="11">
         <f>IF(ISBLANK(A62), "", VLOOKUP($B62, _xlfn.IFS($A62="Solid fuels", $S$9:$Z$28,$A62="Liquid fuels", $S$29:$Z$52,$A62="Light duty vehicles",$S$49:$AA$50,$A62="Heavy duty vehicles",$S$51:$AA$58,$A62="Aviation",$S$59:$AA$61,$A62="Vessel",$S$63:$AA$65,TRUE,$S$66:$AA$66),2,FALSE))</f>

</xml_diff>